<commit_message>
fix(inventory): align GTL lifetime allocation with reference calendar
Adopt the explicitly approved van der Giesen (2014) SI S10/Table S22 reference: 18000 tonnes/day x 300 operating days/year x 30 years. Correct 57 construction doses in seven existing workbooks from 6.7e-12 to 1/(18000*1000*300*30) plant units/kg fuel. Document this as an operating-basis assumption, not measured or future engineering validation. Preserve construction recipes, fuel outputs, allocation keys and other inputs.

Scope: existing supplemental workbook inventories only. Approved as item 9 of ten on 2026-10-18.

Validation: exact edited-cell/ZIP-part scope, formula/cache round-trip and raw no-write ExcelImporter regression. Shared ecoinvent 3.8-3.12 checks are run after the batch; this does not constitute a full scenario rebuild.
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-synfuels-from-FT-from-coal-gasification-with-CCS.xlsx
+++ b/premise/data/additional_inventories/lci-synfuels-from-FT-from-coal-gasification-with-CCS.xlsx
@@ -2103,8 +2103,12 @@
       <c r="A93" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B93" s="8" t="s">
-        <v>42</v>
+      <c r="B93" s="8" t="inlineStr">
+        <is>
+          <t>APPROVED GTL LIFETIME-OUTPUT REFERENCE ASSUMPTION, 2026-10-18. Van der Giesen et al. (2014), DOI 10.1021/es500191g, SI https://doi.org/10.1021/es500191g.s001, page S10 and Table S22, gives 18000 tonnes fuel/day, 300 operating days/year and 30 years. Adopt that published production calendar as the reference for the existing GTL equipment: 1/(18000*1000*300*30) = 6.172839506172839E-12 plant units/kg fuel, replacing the inconsistent transcribed 6.7E-12. USER-APPROVED OPERATING ASSUMPTION: this uses the published reference output/calendar; it does not establish measured operation, future plant duty or complete catalyst coverage. Existing product-allocation keys, fuel output and construction recipe remain unchanged. No new hardware, metal-content factors, credits or primary/secondary shares. Prior references to the former dose or preserved lifetime allocation are superseded only for this coefficient.
+PREVIOUS NOTES (retained as history; the correction above takes precedence):
+Adapted from van der Giesen et al. 2014. LHV: 45 MJ/kg, Formula: C13H18, Density: 7551 kg/m3. Economic allocation between 3 other co-products. Allocation key for this co-product: 6%.</t>
+        </is>
       </c>
     </row>
     <row r="94" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.2">
@@ -2237,7 +2241,7 @@
         <v>39</v>
       </c>
       <c r="B101" s="9">
-        <v>6.7000000000000001E-12</v>
+        <v>6.172839506172839e-12</v>
       </c>
       <c r="C101" s="8" t="s">
         <v>31</v>
@@ -2331,8 +2335,12 @@
       <c r="A110" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B110" s="8" t="s">
-        <v>44</v>
+      <c r="B110" s="8" t="inlineStr">
+        <is>
+          <t>APPROVED GTL LIFETIME-OUTPUT REFERENCE ASSUMPTION, 2026-10-18. Van der Giesen et al. (2014), DOI 10.1021/es500191g, SI https://doi.org/10.1021/es500191g.s001, page S10 and Table S22, gives 18000 tonnes fuel/day, 300 operating days/year and 30 years. Adopt that published production calendar as the reference for the existing GTL equipment: 1/(18000*1000*300*30) = 6.172839506172839E-12 plant units/kg fuel, replacing the inconsistent transcribed 6.7E-12. USER-APPROVED OPERATING ASSUMPTION: this uses the published reference output/calendar; it does not establish measured operation, future plant duty or complete catalyst coverage. Existing product-allocation keys, fuel output and construction recipe remain unchanged. No new hardware, metal-content factors, credits or primary/secondary shares. Prior references to the former dose or preserved lifetime allocation are superseded only for this coefficient.
+PREVIOUS NOTES (retained as history; the correction above takes precedence):
+Adapted from van der Giesen et al. 2014. LHV: 44.5 MJ/kg, Formula: C13H18, Density: 7551 kg/m3. Economic allocation between 3 other co-products. Allocation key for this co-product: 7%.</t>
+        </is>
       </c>
     </row>
     <row r="111" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.2">
@@ -2465,7 +2473,7 @@
         <v>39</v>
       </c>
       <c r="B118" s="9">
-        <v>6.7000000000000001E-12</v>
+        <v>6.172839506172839e-12</v>
       </c>
       <c r="C118" s="8" t="s">
         <v>31</v>
@@ -2559,8 +2567,12 @@
       <c r="A127" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B127" s="8" t="s">
-        <v>45</v>
+      <c r="B127" s="8" t="inlineStr">
+        <is>
+          <t>APPROVED GTL LIFETIME-OUTPUT REFERENCE ASSUMPTION, 2026-10-18. Van der Giesen et al. (2014), DOI 10.1021/es500191g, SI https://doi.org/10.1021/es500191g.s001, page S10 and Table S22, gives 18000 tonnes fuel/day, 300 operating days/year and 30 years. Adopt that published production calendar as the reference for the existing GTL equipment: 1/(18000*1000*300*30) = 6.172839506172839E-12 plant units/kg fuel, replacing the inconsistent transcribed 6.7E-12. USER-APPROVED OPERATING ASSUMPTION: this uses the published reference output/calendar; it does not establish measured operation, future plant duty or complete catalyst coverage. Existing product-allocation keys, fuel output and construction recipe remain unchanged. No new hardware, metal-content factors, credits or primary/secondary shares. Prior references to the former dose or preserved lifetime allocation are superseded only for this coefficient.
+PREVIOUS NOTES (retained as history; the correction above takes precedence):
+Adapted from van der Giesen et al. 2014. LHV: 43.3 MJ/kg, Formula: C13H18, Density: 7551 kg/m3. Economic allocation between 3 other co-products. Allocation key for this co-product: 16%.</t>
+        </is>
       </c>
     </row>
     <row r="128" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.2">
@@ -2693,7 +2705,7 @@
         <v>39</v>
       </c>
       <c r="B135" s="9">
-        <v>6.7000000000000001E-12</v>
+        <v>6.172839506172839e-12</v>
       </c>
       <c r="C135" s="8" t="s">
         <v>31</v>
@@ -2787,8 +2799,12 @@
       <c r="A144" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B144" s="8" t="s">
-        <v>46</v>
+      <c r="B144" s="8" t="inlineStr">
+        <is>
+          <t>APPROVED GTL LIFETIME-OUTPUT REFERENCE ASSUMPTION, 2026-10-18. Van der Giesen et al. (2014), DOI 10.1021/es500191g, SI https://doi.org/10.1021/es500191g.s001, page S10 and Table S22, gives 18000 tonnes fuel/day, 300 operating days/year and 30 years. Adopt that published production calendar as the reference for the existing GTL equipment: 1/(18000*1000*300*30) = 6.172839506172839E-12 plant units/kg fuel, replacing the inconsistent transcribed 6.7E-12. USER-APPROVED OPERATING ASSUMPTION: this uses the published reference output/calendar; it does not establish measured operation, future plant duty or complete catalyst coverage. Existing product-allocation keys, fuel output and construction recipe remain unchanged. No new hardware, metal-content factors, credits or primary/secondary shares. Prior references to the former dose or preserved lifetime allocation are superseded only for this coefficient.
+PREVIOUS NOTES (retained as history; the correction above takes precedence):
+Adapted from van der Giesen et al. 2014. LHV: 40.2 MJ/kg, Formula: C13H18, Density: 7551 kg/m3. Energy-based allocation between 3 other co-products. Allocation key for this co-product: 21%.</t>
+        </is>
       </c>
     </row>
     <row r="145" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.2">
@@ -2921,7 +2937,7 @@
         <v>39</v>
       </c>
       <c r="B152" s="9">
-        <v>6.7000000000000001E-12</v>
+        <v>6.172839506172839e-12</v>
       </c>
       <c r="C152" s="8" t="s">
         <v>31</v>
@@ -3017,8 +3033,12 @@
       <c r="A161" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B161" s="8" t="s">
-        <v>47</v>
+      <c r="B161" s="8" t="inlineStr">
+        <is>
+          <t>APPROVED GTL LIFETIME-OUTPUT REFERENCE ASSUMPTION, 2026-10-18. Van der Giesen et al. (2014), DOI 10.1021/es500191g, SI https://doi.org/10.1021/es500191g.s001, page S10 and Table S22, gives 18000 tonnes fuel/day, 300 operating days/year and 30 years. Adopt that published production calendar as the reference for the existing GTL equipment: 1/(18000*1000*300*30) = 6.172839506172839E-12 plant units/kg fuel, replacing the inconsistent transcribed 6.7E-12. USER-APPROVED OPERATING ASSUMPTION: this uses the published reference output/calendar; it does not establish measured operation, future plant duty or complete catalyst coverage. Existing product-allocation keys, fuel output and construction recipe remain unchanged. No new hardware, metal-content factors, credits or primary/secondary shares. Prior references to the former dose or preserved lifetime allocation are superseded only for this coefficient.
+PREVIOUS NOTES (retained as history; the correction above takes precedence):
+Adapted from van der Giesen et al. 2014. LHV: 45 MJ/kg, Formula: C13H18, Density: 7551 kg/m3. Energy-based allocation between 3 other co-products. Allocation key for this co-product: 18%.</t>
+        </is>
       </c>
     </row>
     <row r="162" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.2">
@@ -3151,7 +3171,7 @@
         <v>39</v>
       </c>
       <c r="B169" s="9">
-        <v>6.7000000000000001E-12</v>
+        <v>6.172839506172839e-12</v>
       </c>
       <c r="C169" s="8" t="s">
         <v>31</v>
@@ -3245,8 +3265,12 @@
       <c r="A178" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B178" s="8" t="s">
-        <v>48</v>
+      <c r="B178" s="8" t="inlineStr">
+        <is>
+          <t>APPROVED GTL LIFETIME-OUTPUT REFERENCE ASSUMPTION, 2026-10-18. Van der Giesen et al. (2014), DOI 10.1021/es500191g, SI https://doi.org/10.1021/es500191g.s001, page S10 and Table S22, gives 18000 tonnes fuel/day, 300 operating days/year and 30 years. Adopt that published production calendar as the reference for the existing GTL equipment: 1/(18000*1000*300*30) = 6.172839506172839E-12 plant units/kg fuel, replacing the inconsistent transcribed 6.7E-12. USER-APPROVED OPERATING ASSUMPTION: this uses the published reference output/calendar; it does not establish measured operation, future plant duty or complete catalyst coverage. Existing product-allocation keys, fuel output and construction recipe remain unchanged. No new hardware, metal-content factors, credits or primary/secondary shares. Prior references to the former dose or preserved lifetime allocation are superseded only for this coefficient.
+PREVIOUS NOTES (retained as history; the correction above takes precedence):
+Adapted from van der Giesen et al. 2014. LHV: 44.5 MJ/kg, Formula: C13H18, Density: 7551 kg/m3. Energy-based allocation between 3 other co-products. Allocation key for this co-product: 24%.</t>
+        </is>
       </c>
     </row>
     <row r="179" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.2">
@@ -3382,7 +3406,7 @@
         <v>39</v>
       </c>
       <c r="B186" s="9">
-        <v>6.7000000000000001E-12</v>
+        <v>6.172839506172839e-12</v>
       </c>
       <c r="C186" s="8" t="s">
         <v>31</v>
@@ -3476,8 +3500,12 @@
       <c r="A195" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B195" s="8" t="s">
-        <v>49</v>
+      <c r="B195" s="8" t="inlineStr">
+        <is>
+          <t>APPROVED GTL LIFETIME-OUTPUT REFERENCE ASSUMPTION, 2026-10-18. Van der Giesen et al. (2014), DOI 10.1021/es500191g, SI https://doi.org/10.1021/es500191g.s001, page S10 and Table S22, gives 18000 tonnes fuel/day, 300 operating days/year and 30 years. Adopt that published production calendar as the reference for the existing GTL equipment: 1/(18000*1000*300*30) = 6.172839506172839E-12 plant units/kg fuel, replacing the inconsistent transcribed 6.7E-12. USER-APPROVED OPERATING ASSUMPTION: this uses the published reference output/calendar; it does not establish measured operation, future plant duty or complete catalyst coverage. Existing product-allocation keys, fuel output and construction recipe remain unchanged. No new hardware, metal-content factors, credits or primary/secondary shares. Prior references to the former dose or preserved lifetime allocation are superseded only for this coefficient.
+PREVIOUS NOTES (retained as history; the correction above takes precedence):
+Adapted from van der Giesen et al. 2014. LHV: 43.3 MJ/kg, Formula: C13H18, Density: 7551 kg/m3. Energy-based allocation between 3 other co-products. Allocation key for this co-product: 37%. Post corrected to preserve carbon balance.</t>
+        </is>
       </c>
     </row>
     <row r="196" spans="1:8" s="8" customFormat="1" x14ac:dyDescent="0.2">
@@ -3610,7 +3638,7 @@
         <v>39</v>
       </c>
       <c r="B203" s="9">
-        <v>6.7000000000000001E-12</v>
+        <v>6.172839506172839e-12</v>
       </c>
       <c r="C203" s="8" t="s">
         <v>31</v>
@@ -3704,8 +3732,12 @@
       <c r="A212" t="s">
         <v>9</v>
       </c>
-      <c r="B212" t="s">
-        <v>92</v>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>APPROVED GTL LIFETIME-OUTPUT REFERENCE ASSUMPTION, 2026-10-18. Van der Giesen et al. (2014), DOI 10.1021/es500191g, SI https://doi.org/10.1021/es500191g.s001, page S10 and Table S22, gives 18000 tonnes fuel/day, 300 operating days/year and 30 years. Adopt that published production calendar as the reference for the existing GTL equipment: 1/(18000*1000*300*30) = 6.172839506172839E-12 plant units/kg fuel, replacing the inconsistent transcribed 6.7E-12. USER-APPROVED OPERATING ASSUMPTION: this uses the published reference output/calendar; it does not establish measured operation, future plant duty or complete catalyst coverage. Existing product-allocation keys, fuel output and construction recipe remain unchanged. No new hardware, metal-content factors, credits or primary/secondary shares. Prior references to the former dose or preserved lifetime allocation are superseded only for this coefficient.
+PREVIOUS NOTES (retained as history; the correction above takes precedence):
+Adapted from A.E.M. van den Oever, D. Costa, M. Messagie, Prospective life cycle assessment of alternatively fueled heavy-duty trucks, Applied Energy, 2023, https://doi.org/10.1016/j.apenergy.2023.120834. Energy-based allocation between 3 other co-products (diesel, wax and C5-C10 olefins). Allocation key for this co-product: 11%. Post corrected to preserve carbon balance.</t>
+        </is>
       </c>
     </row>
     <row r="213" spans="1:7" x14ac:dyDescent="0.2">
@@ -3827,7 +3859,7 @@
         <v>39</v>
       </c>
       <c r="B220" s="3">
-        <v>6.7000000000000001E-12</v>
+        <v>6.172839506172839e-12</v>
       </c>
       <c r="C220" t="s">
         <v>31</v>

</xml_diff>

<commit_message>
fix(inventory): adopt explicit RWGS pair-level lifetime allocation
Apply the approved reference assumption to six construction doses in six workbooks: 2900 kg CO per half-hour is output of the complete two-reactor unit, operated 8000 h/year for 30 years. Set 1/(2900*2*8000*30) = 7.183908045977011e-10 pair units/kg CO instead of 1.93e-9. Source: van der Giesen (2014), SI S7-S8/Table S19, DOI 10.1021/es500191g.s001. Explicitly document that per-vessel simultaneous throughput would halve this dose. Preserve two-vessel construction, catalyst/zeolite recipes and all other flows; no claim of validated plant performance.

Scope: existing supplemental workbook inventories only. Approved as item 10 of ten on 2026-10-18.

Validation: exact edited-cell/ZIP-part scope, formula/cache round-trip and raw no-write ExcelImporter regression. Shared ecoinvent 3.8-3.12 checks are run after the batch; this does not constitute a full scenario rebuild.
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-synfuels-from-FT-from-coal-gasification-with-CCS.xlsx
+++ b/premise/data/additional_inventories/lci-synfuels-from-FT-from-coal-gasification-with-CCS.xlsx
@@ -4174,8 +4174,14 @@
       <c r="A247" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B247" s="8" t="s">
-        <v>90</v>
+      <c r="B247" s="8" t="inlineStr">
+        <is>
+          <t>APPROVED RWGS PAIR-LEVEL THROUGHPUT ASSUMPTION, 2026-10-18. Van der Giesen et al. (2014), DOI 10.1021/es500191g, SI https://doi.org/10.1021/es500191g.s001, pages S7-S8 and Table S19, states 2900 kg CO per 30 minutes, 8000 operating hours/year and 30 years, for construction represented by a two-reactor unit. EXPLICIT USER-APPROVED BOUNDARY ASSUMPTION: treat 2900 kg per 30 minutes as total output of the COMPLETE TWO-REACTOR UNIT, not per vessel. Then 1/(2900*2*8000*30) = 7.183908045977011E-10 pair units/kg CO, replacing the inconsistent 1.93E-9. The source duty/parallel-vessel interpretation remains ambiguous: if both vessels each deliver this throughput, the dose would be half this value. This reference accounting assumption is not proof of industrial performance. Keep the corrected two-vessel steel recipe, catalyst/zeolite lifetime quantities, CO output and other material/energy flows unchanged. Historical dose statements are superseded only for this coefficient. No new recovery credit or primary/secondary split.
+PREVIOUS NOTES (retained as history; the correction above takes precedence):
+Adapted from van der Giesen et al. 2014. Density of syngas: 0.470kg/m3 @1 bar. LHV: 23.9 MJ/kg.
+Here, the CO2 needed (1.57 kg CO2) comes from a redirected amount from the coal gasification process with CCS (which produces 18 kg CO2 per kg H2 if CCS is not applied).
+We do not need to correct the carbon balance because the amount of CO2 not stored underground ends up anyway embodied in the fuel instead (until combustion).</t>
+        </is>
       </c>
     </row>
     <row r="248" spans="1:7" s="8" customFormat="1" ht="16" x14ac:dyDescent="0.2">
@@ -4251,7 +4257,7 @@
         <v>50</v>
       </c>
       <c r="B252" s="9">
-        <v>1.9300000000000002E-9</v>
+        <v>7.183908045977011e-10</v>
       </c>
       <c r="C252" s="8" t="s">
         <v>8</v>

</xml_diff>